<commit_message>
notes for session 2
</commit_message>
<xml_diff>
--- a/materials/introduction.xlsx
+++ b/materials/introduction.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Z:\temp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E550A0B6-8AFD-4B49-9C1F-2F5618A098A8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{476F2C6A-EE33-472A-BEA7-5A6D40DE1B9C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="22365" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21885" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Start" sheetId="4" r:id="rId1"/>
@@ -18,13 +18,14 @@
     <sheet name="with_plot" sheetId="1" r:id="rId3"/>
     <sheet name="simple" sheetId="6" r:id="rId4"/>
     <sheet name="conditional_cost" sheetId="5" r:id="rId5"/>
+    <sheet name="Bike_sales" sheetId="8" r:id="rId6"/>
   </sheets>
   <calcPr calcId="191029"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="97" uniqueCount="34">
   <si>
     <t>April</t>
   </si>
@@ -99,13 +100,40 @@
   </si>
   <si>
     <t>Production &gt;= 130000 =</t>
+  </si>
+  <si>
+    <t>Bike</t>
+  </si>
+  <si>
+    <t>Sales</t>
+  </si>
+  <si>
+    <t>Turnover</t>
+  </si>
+  <si>
+    <t>Cost</t>
+  </si>
+  <si>
+    <t>City-Trip</t>
+  </si>
+  <si>
+    <t>TourenCross</t>
+  </si>
+  <si>
+    <t>MTB-Downhill</t>
+  </si>
+  <si>
+    <t>MTB-SingleTrail</t>
+  </si>
+  <si>
+    <t>MTB-Monster</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -116,6 +144,14 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -125,7 +161,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -151,11 +187,26 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
@@ -177,6 +228,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1289,4 +1344,101 @@
   <pageMargins left="0.78740157499999996" right="0.78740157499999996" top="0.984251969" bottom="0.984251969" header="0.4921259845" footer="0.4921259845"/>
   <headerFooter alignWithMargins="0"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7A600789-C080-4141-B61C-543C0E3F31D0}">
+  <dimension ref="B2:E7"/>
+  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="2" max="2" width="17.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:5" ht="15" x14ac:dyDescent="0.2">
+      <c r="B2" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="C2" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="D2" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="E2" s="9" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="3" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B3" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="C3" s="10">
+        <v>3</v>
+      </c>
+      <c r="D3" s="10">
+        <v>7797</v>
+      </c>
+      <c r="E3" s="10">
+        <v>4410</v>
+      </c>
+    </row>
+    <row r="4" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B4" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="C4" s="10">
+        <v>5</v>
+      </c>
+      <c r="D4" s="10">
+        <v>18995</v>
+      </c>
+      <c r="E4" s="10">
+        <v>12500</v>
+      </c>
+    </row>
+    <row r="5" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B5" s="10" t="s">
+        <v>31</v>
+      </c>
+      <c r="C5" s="10">
+        <v>1</v>
+      </c>
+      <c r="D5" s="10">
+        <v>5799</v>
+      </c>
+      <c r="E5" s="10">
+        <v>4800</v>
+      </c>
+    </row>
+    <row r="6" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B6" s="10" t="s">
+        <v>32</v>
+      </c>
+      <c r="C6" s="10">
+        <v>4</v>
+      </c>
+      <c r="D6" s="10">
+        <v>29996</v>
+      </c>
+      <c r="E6" s="10">
+        <v>19200</v>
+      </c>
+    </row>
+    <row r="7" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B7" s="10" t="s">
+        <v>33</v>
+      </c>
+      <c r="C7" s="10">
+        <v>9</v>
+      </c>
+      <c r="D7" s="10">
+        <v>89910</v>
+      </c>
+      <c r="E7" s="10">
+        <v>75600</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>